<commit_message>
Commit changes from Hands-on Ex10, Take-home Ex03
</commit_message>
<xml_diff>
--- a/Take-home_Ex/Take-home_Ex03/data/StationList.xlsx
+++ b/Take-home_Ex/Take-home_Ex03/data/StationList.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2. SMU - MITB\Term 5\ISSS608 Visual\YX-Leng\ISSS608-VisualAnalytics\Take-home_Ex\Take-home_Ex03\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16FE9BD-602B-4D34-B66D-301F9223F63C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BA3F80-636F-4086-8B5E-850975619E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CDE2D9D4-A969-43A4-8A9B-23E9E88774E8}"/>
+    <workbookView xWindow="37380" yWindow="0" windowWidth="20325" windowHeight="15585" xr2:uid="{CDE2D9D4-A969-43A4-8A9B-23E9E88774E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="95">
   <si>
     <t>S24</t>
   </si>
@@ -144,12 +144,6 @@
     <t>S25</t>
   </si>
   <si>
-    <t>Semakau Island</t>
-  </si>
-  <si>
-    <t>S102</t>
-  </si>
-  <si>
     <t>Sembawang</t>
   </si>
   <si>
@@ -178,6 +172,159 @@
   </si>
   <si>
     <t>StationID</t>
+  </si>
+  <si>
+    <t>Rainfall</t>
+  </si>
+  <si>
+    <t>Bukit Panjang</t>
+  </si>
+  <si>
+    <t>S64</t>
+  </si>
+  <si>
+    <t>Bukit Timah</t>
+  </si>
+  <si>
+    <t>Choa Chu Kang (Central)</t>
+  </si>
+  <si>
+    <t>Jurong Pier</t>
+  </si>
+  <si>
+    <t>Kent Ridge</t>
+  </si>
+  <si>
+    <t>Kranji Reservoir</t>
+  </si>
+  <si>
+    <t>Lim Chu Kang</t>
+  </si>
+  <si>
+    <t>Lower Peirce Reservoir</t>
+  </si>
+  <si>
+    <t>Macritchie Reservoir</t>
+  </si>
+  <si>
+    <t>Mandai</t>
+  </si>
+  <si>
+    <t>Marine Parade</t>
+  </si>
+  <si>
+    <t>Nicoll Highway</t>
+  </si>
+  <si>
+    <t>Pasir Ris (Central)</t>
+  </si>
+  <si>
+    <t>Pasir Ris (West)</t>
+  </si>
+  <si>
+    <t>Punggol</t>
+  </si>
+  <si>
+    <t>Queenstown</t>
+  </si>
+  <si>
+    <t>Simei</t>
+  </si>
+  <si>
+    <t>Somerset (Road)</t>
+  </si>
+  <si>
+    <t>Tanjong Katong</t>
+  </si>
+  <si>
+    <t>Toa Payoh</t>
+  </si>
+  <si>
+    <t>Tuas</t>
+  </si>
+  <si>
+    <t>Ulu Pandan</t>
+  </si>
+  <si>
+    <t>Upper Peirce Reservoir</t>
+  </si>
+  <si>
+    <t>Whampoa</t>
+  </si>
+  <si>
+    <t>Buona Vista</t>
+  </si>
+  <si>
+    <t>S90</t>
+  </si>
+  <si>
+    <t>S92</t>
+  </si>
+  <si>
+    <t>S114</t>
+  </si>
+  <si>
+    <t>S33</t>
+  </si>
+  <si>
+    <t>S71</t>
+  </si>
+  <si>
+    <t>S66</t>
+  </si>
+  <si>
+    <t>S112</t>
+  </si>
+  <si>
+    <t>S08</t>
+  </si>
+  <si>
+    <t>S07</t>
+  </si>
+  <si>
+    <t>S40</t>
+  </si>
+  <si>
+    <t>S113</t>
+  </si>
+  <si>
+    <t>S119</t>
+  </si>
+  <si>
+    <t>S94</t>
+  </si>
+  <si>
+    <t>S29</t>
+  </si>
+  <si>
+    <t>S81</t>
+  </si>
+  <si>
+    <t>S77</t>
+  </si>
+  <si>
+    <t>S84</t>
+  </si>
+  <si>
+    <t>S79</t>
+  </si>
+  <si>
+    <t>S78</t>
+  </si>
+  <si>
+    <t>S88</t>
+  </si>
+  <si>
+    <t>S89</t>
+  </si>
+  <si>
+    <t>S35</t>
+  </si>
+  <si>
+    <t>S69</t>
+  </si>
+  <si>
+    <t>S123</t>
   </si>
 </sst>
 </file>
@@ -549,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A995077D-BA74-427E-B81B-B588DC35B494}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -560,19 +707,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" t="s">
         <v>43</v>
       </c>
-      <c r="B1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1" t="s">
-        <v>45</v>
-      </c>
       <c r="D1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -611,53 +758,53 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="D4">
-        <v>1.3677999999999999</v>
+        <v>1.3823000000000001</v>
       </c>
       <c r="E4">
-        <v>103.9823</v>
+        <v>103.7607</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="D5">
-        <v>1.3729</v>
+        <v>1.3190999999999999</v>
       </c>
       <c r="E5">
-        <v>103.72239999999999</v>
+        <v>103.8193</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="D6">
-        <v>1.3318000000000001</v>
+        <v>1.2841</v>
       </c>
       <c r="E6">
-        <v>103.7762</v>
+        <v>103.78879999999999</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -665,33 +812,33 @@
         <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>1.3132999999999999</v>
+        <v>1.3677999999999999</v>
       </c>
       <c r="E7">
-        <v>103.962</v>
+        <v>103.9823</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>2</v>
+        <v>73</v>
       </c>
       <c r="D8">
-        <v>1.3458000000000001</v>
+        <v>1.3821000000000001</v>
       </c>
       <c r="E8">
-        <v>103.68170000000001</v>
+        <v>103.7381</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -699,16 +846,16 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D9">
-        <v>1.2542</v>
+        <v>1.3729</v>
       </c>
       <c r="E9">
-        <v>103.6741</v>
+        <v>103.72239999999999</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -716,16 +863,16 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D10">
-        <v>1.2799</v>
+        <v>1.3318000000000001</v>
       </c>
       <c r="E10">
-        <v>103.8703</v>
+        <v>103.7762</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -733,16 +880,16 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D11">
-        <v>1.3106</v>
+        <v>1.3132999999999999</v>
       </c>
       <c r="E11">
-        <v>103.8365</v>
+        <v>103.962</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -750,16 +897,16 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D12">
-        <v>1.2824</v>
+        <v>1.3458000000000001</v>
       </c>
       <c r="E12">
-        <v>103.75449999999999</v>
+        <v>103.68170000000001</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -767,135 +914,135 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="D13">
-        <v>1.3571</v>
+        <v>1.2542</v>
       </c>
       <c r="E13">
-        <v>103.9037</v>
+        <v>103.6741</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
-        <v>6</v>
+        <v>74</v>
       </c>
       <c r="D14">
-        <v>1.4168000000000001</v>
+        <v>1.3082</v>
       </c>
       <c r="E14">
-        <v>103.96729999999999</v>
+        <v>103.71</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="D15">
-        <v>1.4167000000000001</v>
+        <v>1.2923</v>
       </c>
       <c r="E15">
-        <v>103.86499999999999</v>
+        <v>103.78149999999999</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="D16">
-        <v>1.1901999999999999</v>
+        <v>1.4387000000000001</v>
       </c>
       <c r="E16">
-        <v>103.7657</v>
+        <v>103.736</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="D17">
-        <v>1.425</v>
+        <v>1.4388000000000001</v>
       </c>
       <c r="E17">
-        <v>103.82</v>
+        <v>103.7017</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="C18" t="s">
-        <v>4</v>
+        <v>78</v>
       </c>
       <c r="D18">
-        <v>1.2503</v>
+        <v>1.37</v>
       </c>
       <c r="E18">
-        <v>103.8275</v>
+        <v>103.8271</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C19" t="s">
-        <v>1</v>
+        <v>79</v>
       </c>
       <c r="D19">
-        <v>1.3406</v>
+        <v>1.3418000000000001</v>
       </c>
       <c r="E19">
-        <v>103.8882</v>
+        <v>103.8339</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="D20">
-        <v>1.3857999999999999</v>
+        <v>1.4067000000000001</v>
       </c>
       <c r="E20">
-        <v>103.7119</v>
+        <v>103.78319999999999</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -903,19 +1050,432 @@
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21">
+        <v>1.2799</v>
+      </c>
+      <c r="E21">
+        <v>103.8703</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22">
+        <v>1.3049999999999999</v>
+      </c>
+      <c r="E22">
+        <v>103.91119999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23">
+        <v>1.3106</v>
+      </c>
+      <c r="E23">
+        <v>103.8365</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24">
+        <v>1.2949999999999999</v>
+      </c>
+      <c r="E24">
+        <v>103.8622</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25">
+        <v>1.2824</v>
+      </c>
+      <c r="E25">
+        <v>103.75449999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" t="s">
+        <v>83</v>
+      </c>
+      <c r="D26">
+        <v>1.3678999999999999</v>
+      </c>
+      <c r="E26">
+        <v>103.94889999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" t="s">
+        <v>84</v>
+      </c>
+      <c r="D27">
+        <v>1.3865000000000001</v>
+      </c>
+      <c r="E27">
+        <v>103.9413</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" t="s">
+        <v>29</v>
+      </c>
+      <c r="D28">
+        <v>1.3571</v>
+      </c>
+      <c r="E28">
+        <v>103.9037</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>1.4168000000000001</v>
+      </c>
+      <c r="E29">
+        <v>103.96729999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" t="s">
+        <v>85</v>
+      </c>
+      <c r="D30">
+        <v>1.4028</v>
+      </c>
+      <c r="E30">
+        <v>103.90949999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31">
+        <v>1.2937000000000001</v>
+      </c>
+      <c r="E31">
+        <v>103.81270000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" t="s">
+        <v>33</v>
+      </c>
+      <c r="D32">
+        <v>1.4167000000000001</v>
+      </c>
+      <c r="E32">
+        <v>103.86499999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" t="s">
+        <v>35</v>
+      </c>
+      <c r="D33">
+        <v>1.425</v>
+      </c>
+      <c r="E33">
+        <v>103.82</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" t="s">
+        <v>31</v>
+      </c>
+      <c r="C34" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34">
+        <v>1.2503</v>
+      </c>
+      <c r="E34">
+        <v>103.8275</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" t="s">
+        <v>62</v>
+      </c>
+      <c r="C35" t="s">
+        <v>87</v>
+      </c>
+      <c r="D35">
+        <v>1.3443000000000001</v>
+      </c>
+      <c r="E35">
+        <v>103.94410000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36">
+        <v>1.3003</v>
+      </c>
+      <c r="E36">
+        <v>103.8372</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>1.3406</v>
+      </c>
+      <c r="E37">
+        <v>103.8882</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" t="s">
+        <v>64</v>
+      </c>
+      <c r="C38" t="s">
+        <v>89</v>
+      </c>
+      <c r="D38">
+        <v>1.3069999999999999</v>
+      </c>
+      <c r="E38">
+        <v>103.8907</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C39" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39">
+        <v>1.3857999999999999</v>
+      </c>
+      <c r="E39">
+        <v>103.7119</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" t="s">
+        <v>90</v>
+      </c>
+      <c r="D40">
+        <v>1.3416999999999999</v>
+      </c>
+      <c r="E40">
+        <v>103.8515</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" t="s">
+        <v>91</v>
+      </c>
+      <c r="D41">
+        <v>1.3199000000000001</v>
+      </c>
+      <c r="E41">
+        <v>103.6613</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>18</v>
+      </c>
+      <c r="B42" t="s">
+        <v>38</v>
+      </c>
+      <c r="C42" t="s">
         <v>13</v>
       </c>
-      <c r="D21">
+      <c r="D42">
         <v>1.2938000000000001</v>
       </c>
-      <c r="E21">
+      <c r="E42">
         <v>103.61839999999999</v>
       </c>
     </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43" t="s">
+        <v>67</v>
+      </c>
+      <c r="C43" t="s">
+        <v>92</v>
+      </c>
+      <c r="D43">
+        <v>1.3325</v>
+      </c>
+      <c r="E43">
+        <v>103.755</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44" t="s">
+        <v>68</v>
+      </c>
+      <c r="C44" t="s">
+        <v>93</v>
+      </c>
+      <c r="D44">
+        <v>1.3704000000000001</v>
+      </c>
+      <c r="E44">
+        <v>103.80459999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>69</v>
+      </c>
+      <c r="C45" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45">
+        <v>1.3213999999999999</v>
+      </c>
+      <c r="E45">
+        <v>103.85769999999999</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{A995077D-BA74-427E-B81B-B588DC35B494}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F45">
+      <sortCondition ref="B1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>